<commit_message>
Add governed Excel onboarding import
</commit_message>
<xml_diff>
--- a/public/downloads/AiFrogi-Simple-AI-Bot-Onboarding.xlsx
+++ b/public/downloads/AiFrogi-Simple-AI-Bot-Onboarding.xlsx
@@ -2,7 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Bot Setup" sheetId="1" r:id="Ra3a67af330014fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Bot Setup" sheetId="1" r:id="R17e2a6a071ae48a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved FAQs" sheetId="2" r:id="Rebb64d6cb8e44825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Sources" sheetId="3" r:id="R487731ce3edf48ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="18">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -112,8 +114,14 @@
       <x:color rgb="FFE2C66D"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF5F5A52"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -150,6 +158,21 @@
         <x:fgColor rgb="FF101010"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF151515"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDE9DF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="12">
     <x:border/>
@@ -263,7 +286,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="87">
+  <x:cellXfs count="95">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -476,6 +499,20 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -772,11 +809,11 @@
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="77" t="str">
-        <x:v>Mobile / WhatsApp *</x:v>
+        <x:v>Mobile number *</x:v>
       </x:c>
       <x:c r="B12" s="78"/>
       <x:c r="C12" s="79" t="str">
-        <x:v>Include country code</x:v>
+        <x:v>Include country code; do not enter OTPs or passwords</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -913,10 +950,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B28" s="74" t="str">
-        <x:v>Email this completed Excel file</x:v>
+        <x:v>Validate and preview</x:v>
       </x:c>
       <x:c r="C28" s="76" t="str">
-        <x:v>Send to info@aifrogi.com with approved brochures or documents.</x:v>
+        <x:v>Sign in to AiFrogi and upload this completed workbook.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
@@ -924,10 +961,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B29" s="77" t="str">
-        <x:v>AiFrogi prepares your bot</x:v>
+        <x:v>Import approved information</x:v>
       </x:c>
       <x:c r="C29" s="79" t="str">
-        <x:v>We structure approved knowledge, persona, safety limits and handover.</x:v>
+        <x:v>Business details are updated and FAQs are staged inside Intelligence.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
@@ -935,10 +972,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B30" s="77" t="str">
-        <x:v>You review the preview</x:v>
+        <x:v>Review real answers</x:v>
       </x:c>
       <x:c r="C30" s="79" t="str">
-        <x:v>Confirm the bot's real answers before installation.</x:v>
+        <x:v>Approve each field and conversational preview before publication.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
@@ -965,4 +1002,187 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="88" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="B1" s="88" t="str">
+        <x:v>Customer question</x:v>
+      </x:c>
+      <x:c r="C1" s="88" t="str">
+        <x:v>Approved answer</x:v>
+      </x:c>
+      <x:c r="D1" s="88" t="str">
+        <x:v>Refresh days</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="91" t="str">
+        <x:v>Contact</x:v>
+      </x:c>
+      <x:c r="B2" s="91" t="str">
+        <x:v>How can I contact your team?</x:v>
+      </x:c>
+      <x:c r="C2" s="91" t="str">
+        <x:v>Replace this with the approved public phone and email.</x:v>
+      </x:c>
+      <x:c r="D2" s="91" t="n">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="91" t="str">
+        <x:v>Services</x:v>
+      </x:c>
+      <x:c r="B3" s="91" t="str">
+        <x:v>What services do you provide?</x:v>
+      </x:c>
+      <x:c r="C3" s="91" t="str">
+        <x:v>Replace this with a short approved answer.</x:v>
+      </x:c>
+      <x:c r="D3" s="91" t="n">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="91" t="str">
+        <x:v>Pricing</x:v>
+      </x:c>
+      <x:c r="B4" s="91" t="str">
+        <x:v>How much does it cost?</x:v>
+      </x:c>
+      <x:c r="C4" s="91" t="str">
+        <x:v>Replace this only with an approved price or explain how to request a quote.</x:v>
+      </x:c>
+      <x:c r="D4" s="91" t="n">
+        <x:v>30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="91" t="str">
+        <x:v>Hours</x:v>
+      </x:c>
+      <x:c r="B5" s="91" t="str">
+        <x:v>When are you open?</x:v>
+      </x:c>
+      <x:c r="C5" s="91" t="str">
+        <x:v>Replace this with approved business hours and timezone.</x:v>
+      </x:c>
+      <x:c r="D5" s="91" t="n">
+        <x:v>30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="91" t="str">
+        <x:v>Location</x:v>
+      </x:c>
+      <x:c r="B6" s="91" t="str">
+        <x:v>Where are you located?</x:v>
+      </x:c>
+      <x:c r="C6" s="91" t="str">
+        <x:v>Replace this with the approved address or map link.</x:v>
+      </x:c>
+      <x:c r="D6" s="91" t="n">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7"/>
+      <x:c r="B7"/>
+      <x:c r="C7"/>
+      <x:c r="D7"/>
+    </x:row>
+    <x:row r="8" ht="38" customHeight="1">
+      <x:c r="A8" s="94" t="str">
+        <x:v>Add more rows below. Do not include passwords, OTPs, secret keys, unapproved promises or sensitive personal data.</x:v>
+      </x:c>
+      <x:c r="B8"/>
+      <x:c r="C8"/>
+      <x:c r="D8"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A8:D8"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="88" t="str">
+        <x:v>Source type</x:v>
+      </x:c>
+      <x:c r="B1" s="88" t="str">
+        <x:v>Approved URL or file name</x:v>
+      </x:c>
+      <x:c r="C1" s="88" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="91" t="str">
+        <x:v>Website</x:v>
+      </x:c>
+      <x:c r="B2" s="91" t="str">
+        <x:v>https://yourbusiness.com</x:v>
+      </x:c>
+      <x:c r="C2" s="91" t="str">
+        <x:v>Only add pages the bot is allowed to use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="91" t="str">
+        <x:v>Policy</x:v>
+      </x:c>
+      <x:c r="B3" s="91" t="str">
+        <x:v>refund-policy.pdf</x:v>
+      </x:c>
+      <x:c r="C3" s="91" t="str">
+        <x:v>Upload the file separately in Intelligence after import.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4"/>
+      <x:c r="B4"/>
+      <x:c r="C4"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5"/>
+      <x:c r="B5"/>
+      <x:c r="C5"/>
+    </x:row>
+    <x:row r="6" ht="38" customHeight="1">
+      <x:c r="A6" s="94" t="str">
+        <x:v>These entries are references only. AiFrogi never publishes a source or answer without authorised review.</x:v>
+      </x:c>
+      <x:c r="B6"/>
+      <x:c r="C6"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A6:C6"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>